<commit_message>
Fix ICD9 fuzzy matching: filter out non-oral/cranial RC053 entries (stomach, intestinal, etc.)
Agent-Logs-Url: https://github.com/AmyLiSiHan/ICD/sessions/34e41b2c-cbdb-43dd-baf5-5861157d894e

Co-authored-by: AmyLiSiHan <245517736+AmyLiSiHan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/icd10.xlsx
+++ b/icd10.xlsx
@@ -11411,12 +11411,12 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>04.8106</t>
+          <t>04.8101</t>
         </is>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>股神经阻滞术</t>
+          <t>周围神经阻滞术</t>
         </is>
       </c>
       <c r="G2" s="0" t="inlineStr">
@@ -11439,12 +11439,12 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>04.8106</t>
+          <t>04.8101</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>股神经阻滞术</t>
+          <t>周围神经阻滞术</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
@@ -11581,12 +11581,12 @@
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>04.8106</t>
+          <t>04.8101</t>
         </is>
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>股神经阻滞术</t>
+          <t>周围神经阻滞术</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
@@ -11783,17 +11783,17 @@
       </c>
       <c r="D15" s="0" t="inlineStr">
         <is>
-          <t>44.2201</t>
+          <t>22.1100x002</t>
         </is>
       </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
-          <t>内镜下幽门球囊扩张术</t>
+          <t>鼻内窥镜下鼻窦活检</t>
         </is>
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>治疗性操作</t>
+          <t>诊断性操作</t>
         </is>
       </c>
     </row>
@@ -11953,17 +11953,17 @@
       </c>
       <c r="D21" s="0" t="inlineStr">
         <is>
-          <t>45.3305</t>
+          <t>22.1100x002</t>
         </is>
       </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
-          <t>内镜下小肠病损切除术</t>
+          <t>鼻内窥镜下鼻窦活检</t>
         </is>
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>治疗性操作</t>
+          <t>诊断性操作</t>
         </is>
       </c>
     </row>
@@ -11981,12 +11981,12 @@
       </c>
       <c r="D22" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>22.0100x003</t>
         </is>
       </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>上颌窦穿刺抽吸灌洗</t>
         </is>
       </c>
       <c r="G22" s="0" t="inlineStr">
@@ -12065,12 +12065,12 @@
       </c>
       <c r="D25" s="0" t="inlineStr">
         <is>
-          <t>23.0100</t>
+          <t>23.0900</t>
         </is>
       </c>
       <c r="F25" s="0" t="inlineStr">
         <is>
-          <t>拔除乳牙</t>
+          <t>拔除其他牙</t>
         </is>
       </c>
       <c r="G25" s="0" t="inlineStr">
@@ -12121,12 +12121,12 @@
       </c>
       <c r="D27" s="0" t="inlineStr">
         <is>
-          <t>23.7001</t>
+          <t>23.7000x001</t>
         </is>
       </c>
       <c r="F27" s="0" t="inlineStr">
         <is>
-          <t>牙髓切除术</t>
+          <t>牙神经摘除术</t>
         </is>
       </c>
       <c r="G27" s="0" t="inlineStr">
@@ -12177,12 +12177,12 @@
       </c>
       <c r="D29" s="0" t="inlineStr">
         <is>
-          <t>23.7001</t>
+          <t>23.7000x001</t>
         </is>
       </c>
       <c r="F29" s="0" t="inlineStr">
         <is>
-          <t>牙髓切除术</t>
+          <t>牙神经摘除术</t>
         </is>
       </c>
       <c r="G29" s="0" t="inlineStr">
@@ -12613,12 +12613,12 @@
       </c>
       <c r="D44" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>25.1x04</t>
         </is>
       </c>
       <c r="F44" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>支撑喉镜下舌根部病损切除术</t>
         </is>
       </c>
       <c r="G44" s="0" t="inlineStr">
@@ -12727,12 +12727,12 @@
       </c>
       <c r="D48" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>25.1x04</t>
         </is>
       </c>
       <c r="F48" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>支撑喉镜下舌根部病损切除术</t>
         </is>
       </c>
       <c r="G48" s="0" t="inlineStr">
@@ -12757,12 +12757,12 @@
       </c>
       <c r="D49" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>25.1x04</t>
         </is>
       </c>
       <c r="F49" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>支撑喉镜下舌根部病损切除术</t>
         </is>
       </c>
       <c r="G49" s="0" t="inlineStr">
@@ -12787,12 +12787,12 @@
       </c>
       <c r="D50" s="0" t="inlineStr">
         <is>
-          <t>23.7001</t>
+          <t>24.7x02</t>
         </is>
       </c>
       <c r="F50" s="0" t="inlineStr">
         <is>
-          <t>牙髓切除术</t>
+          <t>牙钢丝矫形术</t>
         </is>
       </c>
       <c r="G50" s="0" t="inlineStr">
@@ -12877,12 +12877,12 @@
       </c>
       <c r="D53" s="0" t="inlineStr">
         <is>
-          <t>23.7001</t>
+          <t>24.7x02</t>
         </is>
       </c>
       <c r="F53" s="0" t="inlineStr">
         <is>
-          <t>牙髓切除术</t>
+          <t>牙钢丝矫形术</t>
         </is>
       </c>
       <c r="G53" s="0" t="inlineStr">
@@ -12907,12 +12907,12 @@
       </c>
       <c r="D54" s="0" t="inlineStr">
         <is>
-          <t>23.7001</t>
+          <t>24.7x02</t>
         </is>
       </c>
       <c r="F54" s="0" t="inlineStr">
         <is>
-          <t>牙髓切除术</t>
+          <t>牙钢丝矫形术</t>
         </is>
       </c>
       <c r="G54" s="0" t="inlineStr">
@@ -13231,12 +13231,12 @@
       </c>
       <c r="D65" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>25.1x04</t>
         </is>
       </c>
       <c r="F65" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>支撑喉镜下舌根部病损切除术</t>
         </is>
       </c>
       <c r="G65" s="0" t="inlineStr">
@@ -13259,17 +13259,17 @@
       </c>
       <c r="D66" s="0" t="inlineStr">
         <is>
-          <t>51.8806</t>
+          <t>26.9101</t>
         </is>
       </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
-          <t>胆道镜下胆管结石取出术</t>
+          <t>腮腺导管探查术</t>
         </is>
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>治疗性操作</t>
+          <t>诊断性操作</t>
         </is>
       </c>
     </row>
@@ -13287,17 +13287,17 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>26.9101</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>腮腺导管探查术</t>
         </is>
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>治疗性操作</t>
+          <t>诊断性操作</t>
         </is>
       </c>
     </row>
@@ -13315,17 +13315,17 @@
       </c>
       <c r="D68" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>26.9101</t>
         </is>
       </c>
       <c r="F68" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>腮腺导管探查术</t>
         </is>
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>治疗性操作</t>
+          <t>诊断性操作</t>
         </is>
       </c>
     </row>
@@ -13907,12 +13907,12 @@
       </c>
       <c r="D89" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>27.4907</t>
         </is>
       </c>
       <c r="F89" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>口病损射频消融术</t>
         </is>
       </c>
       <c r="G89" s="0" t="inlineStr">
@@ -14413,12 +14413,12 @@
       </c>
       <c r="D107" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>76.7300</t>
         </is>
       </c>
       <c r="F107" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>上颌骨骨折闭合性复位术</t>
         </is>
       </c>
       <c r="G107" s="0" t="inlineStr">
@@ -14443,12 +14443,12 @@
       </c>
       <c r="D108" s="0" t="inlineStr">
         <is>
-          <t>43.4100x014</t>
+          <t>76.7500</t>
         </is>
       </c>
       <c r="F108" s="0" t="inlineStr">
         <is>
-          <t>胃镜下胃病损切除术</t>
+          <t>下颌骨骨折闭合性复位术</t>
         </is>
       </c>
       <c r="G108" s="0" t="inlineStr">
@@ -14555,12 +14555,12 @@
       </c>
       <c r="D112" s="0" t="inlineStr">
         <is>
-          <t>43.4105</t>
+          <t>76.7500</t>
         </is>
       </c>
       <c r="F112" s="0" t="inlineStr">
         <is>
-          <t>内镜下胃息肉切除术</t>
+          <t>下颌骨骨折闭合性复位术</t>
         </is>
       </c>
       <c r="G112" s="0" t="inlineStr">
@@ -14667,12 +14667,12 @@
       </c>
       <c r="D116" s="0" t="inlineStr">
         <is>
-          <t>43.4105</t>
+          <t>76.7300</t>
         </is>
       </c>
       <c r="F116" s="0" t="inlineStr">
         <is>
-          <t>内镜下胃息肉切除术</t>
+          <t>上颌骨骨折闭合性复位术</t>
         </is>
       </c>
       <c r="G116" s="0" t="inlineStr">

</xml_diff>